<commit_message>
auto: session 2026-08-17 17:53
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/File báo giá - lần 2 (Giáo dục, PR cá nhân, PR công ty, Emagazine).xlsx
+++ b/File báo giá - lần 2 (Giáo dục, PR cá nhân, PR công ty, Emagazine).xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -92,13 +97,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -115,6 +120,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -495,11 +503,12 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="90" customHeight="1">
+    <row r="3" ht="130" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Cơ chế giá giữ nguyên như báo giá lần 1: đây là giá vốn Digicom đàm phán trực tiếp với nhà cung cấp (không cộng thêm phí trung gian), đã kiểm tra đối chiếu từng đầu báo trước khi gửi. Danh sách lần này đầy đủ hơn - bổ sung nhóm Giáo dục, tách riêng PR cá nhân và PR công ty để dễ chọn theo đúng mục đích, và thêm lựa chọn bài Emagazine (định dạng dài, thiết kế media riêng, hiệu ứng chuyển động) cho nhu cầu truyền thông cao cấp.
-Ưu đãi: đặt từ 3 đầu báo trở lên trong đơn - tặng kèm viết bài chuẩn SEO miễn phí (không tính thêm phí viết bài cho các báo đó) và được tư vấn/chọn báo miễn phí, không ràng buộc.</t>
+          <t>Công thức giá: giá vốn DanaSEO hiện hành TRỪ THÊM 5% (chốt riêng cho khách này). Các báo lấy nguồn từ NCC khác DanaSEO (Brando, Xuyên Việt Media, Admicro, Rise Media) không có mức giá DanaSEO để đối chiếu -5%, nên giữ nguyên giá vốn gốc từ NCC đó - đã ghi rõ trong cột Nguồn/Ghi chú.
+LƯU Ý QUAN TRỌNG: đối chiếu với 14 báo đã gửi ở báo giá lần 1 (giá = ĐÚNG BẰNG giá vốn DanaSEO, KHÔNG trừ %), phát hiện 8 dòng trong sheet 'PR Công ty' và 2 dòng khác (Kenh14 - sheet Giáo dục, Soha - sheet PR cá nhân) TRÙNG outlet/vị trí đã gửi lần 1. Áp công thức -5% mới thì các dòng này thấp hơn giá đã gửi khách - đã đánh dấu ⚠ trong cột Nguồn/Ghi chú kèm giá cũ để Hiếu quyết định báo lại giá mới cho khách hay giữ nguyên giá đã chốt ở lần 1.
+Ưu đãi: đặt từ 3 đầu báo trở lên trong đơn - tặng kèm viết bài chuẩn SEO miễn phí và tư vấn/chọn báo miễn phí.</t>
         </is>
       </c>
     </row>
@@ -513,33 +522,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1. Ngành Giáo dục - báo/chuyên mục phù hợp PR trường học, trung tâm đào tạo, sản phẩm giáo dục</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2. PR Cá nhân - báo/chuyên mục phù hợp xây dựng thương hiệu cá nhân, KOL, chuyên gia</t>
+          <t>1. Ngành Giáo dục   2. PR Cá nhân   3. PR Công ty   4. Emagazine (bổ sung)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>3. PR Công ty - báo/chuyên mục phù hợp PR doanh nghiệp, sản phẩm, thương hiệu công ty</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>4. Emagazine (bổ sung) - định dạng bài dài cao cấp, thiết kế riêng, hiệu ứng chuyển động</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Liên hệ: 0988 769 317 | info@digicomvn.com | Digito Combat Communication Services Co., Ltd</t>
         </is>
@@ -562,8 +550,8 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -573,10 +561,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Giá niêm yết trực tiếp từ nhà cung cấp báo (đã là giá tốt nhất Digicom đàm phán được, chưa gồm VAT 8% trừ khi ghi chú khác). Giá có thể thay đổi vào phút chót theo chính sách toà soạn - Digicom sẽ báo lại nếu có biến động trước khi khách chốt đăng.</t>
+          <t>Giá = giá vốn DanaSEO hiện hành TRỪ THÊM 5% (đúng công thức Hiếu chốt cho khách này). Với báo lấy nguồn từ NCC khác DanaSEO (không có mức giá DanaSEO để đối chiếu) - giữ nguyên giá vốn gốc, có ghi rõ nguồn. Dòng có ⚠ = TRÙNG outlet/vị trí đã gửi trong báo giá lần 1 nhưng giá SAU khi trừ 5% THẤP HƠN giá đã gửi lần 1 - cần Hiếu xác nhận có báo lại giá mới cho khách hay giữ nguyên giá cũ đã gửi.</t>
         </is>
       </c>
     </row>
@@ -617,7 +605,7 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>5400000</v>
+        <v>5130000</v>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
@@ -626,7 +614,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Cơ quan của Bộ GD&amp;ĐT - đúng chuyên trang giáo dục</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -640,7 +628,7 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>1500000</v>
+        <v>1425000</v>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
@@ -649,7 +637,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Ấn phẩm địa phương của Giáo dục &amp; Thời đại</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -663,14 +651,18 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>3800000</v>
+        <v>3610000</v>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 5 ảnh, 3 link nofollow</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr"/>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
@@ -682,14 +674,18 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>5200000</v>
+        <v>4940000</v>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 5 ảnh, 3 link nofollow</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -701,14 +697,18 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>9200000</v>
+        <v>8740000</v>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, 2 link nofollow</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr"/>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -720,14 +720,18 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>3700000</v>
+        <v>3515000</v>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 7 ảnh, 1 link nofollow</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr"/>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 3,700,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -748,7 +752,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Nguồn: Brando Agency</t>
+          <t>Nguồn: Brando Agency (không phải DanaSEO - giữ nguyên giá vốn, KHÔNG áp công thức -5%)</t>
         </is>
       </c>
     </row>
@@ -771,7 +775,7 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Nguồn: Xuyên Việt Media</t>
+          <t>Nguồn: Xuyên Việt Media (không phải DanaSEO - giữ nguyên giá vốn, KHÔNG áp công thức -5%)</t>
         </is>
       </c>
     </row>
@@ -796,8 +800,8 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -807,10 +811,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Giá niêm yết trực tiếp từ nhà cung cấp báo (đã là giá tốt nhất Digicom đàm phán được, chưa gồm VAT 8% trừ khi ghi chú khác). Giá có thể thay đổi vào phút chót theo chính sách toà soạn - Digicom sẽ báo lại nếu có biến động trước khi khách chốt đăng.</t>
+          <t>Giá = giá vốn DanaSEO hiện hành TRỪ THÊM 5% (đúng công thức Hiếu chốt cho khách này). Với báo lấy nguồn từ NCC khác DanaSEO (không có mức giá DanaSEO để đối chiếu) - giữ nguyên giá vốn gốc, có ghi rõ nguồn. Dòng có ⚠ = TRÙNG outlet/vị trí đã gửi trong báo giá lần 1 nhưng giá SAU khi trừ 5% THẤP HƠN giá đã gửi lần 1 - cần Hiếu xác nhận có báo lại giá mới cho khách hay giữ nguyên giá cũ đã gửi.</t>
         </is>
       </c>
     </row>
@@ -851,7 +855,7 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>6100000</v>
+        <v>5795000</v>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
@@ -860,7 +864,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Phù hợp PR chuyên gia, KOL trẻ, ẩm thực/giải trí</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -874,7 +878,7 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>6800000</v>
+        <v>6460000</v>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
@@ -883,7 +887,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Phù hợp PR làm đẹp, thời trang cá nhân</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -897,7 +901,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>10200000</v>
+        <v>9690000</v>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
@@ -906,7 +910,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Vị trí nổi bật nhất Kenh14</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -920,14 +924,18 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>4600000</v>
+        <v>4370000</v>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 5 ảnh, 1 link nofollow</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr"/>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 4,600,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -939,7 +947,7 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>3700000</v>
+        <v>3515000</v>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
@@ -948,7 +956,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Báo phụ nữ - phù hợp PR cá nhân nữ giới</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -962,7 +970,7 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>3800000</v>
+        <v>3610000</v>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
@@ -971,7 +979,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Báo gia đình - phù hợp xây hình ảnh cá nhân đời thường</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -985,7 +993,7 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>3200000</v>
+        <v>3040000</v>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
@@ -994,7 +1002,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Báo giải trí - phù hợp PR nghệ sĩ, người có ảnh hưởng</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -1008,14 +1016,18 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>5000000</v>
+        <v>4750000</v>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, 2 link redirect</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
@@ -1027,7 +1039,7 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>9100000</v>
+        <v>8645000</v>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
@@ -1036,7 +1048,7 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Tạp chí phong cách sống - định vị hình ảnh cao cấp</t>
+          <t>DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -1050,14 +1062,18 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>7400000</v>
+        <v>7030000</v>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, 2 link nofollow</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr"/>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1080,8 +1096,8 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1091,10 +1107,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Giá niêm yết trực tiếp từ nhà cung cấp báo (đã là giá tốt nhất Digicom đàm phán được, chưa gồm VAT 8% trừ khi ghi chú khác). Giá có thể thay đổi vào phút chót theo chính sách toà soạn - Digicom sẽ báo lại nếu có biến động trước khi khách chốt đăng.</t>
+          <t>Giá = giá vốn DanaSEO hiện hành TRỪ THÊM 5% (đúng công thức Hiếu chốt cho khách này). Với báo lấy nguồn từ NCC khác DanaSEO (không có mức giá DanaSEO để đối chiếu) - giữ nguyên giá vốn gốc, có ghi rõ nguồn. Dòng có ⚠ = TRÙNG outlet/vị trí đã gửi trong báo giá lần 1 nhưng giá SAU khi trừ 5% THẤP HƠN giá đã gửi lần 1 - cần Hiếu xác nhận có báo lại giá mới cho khách hay giữ nguyên giá cũ đã gửi.</t>
         </is>
       </c>
     </row>
@@ -1135,14 +1151,18 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>5400000</v>
+        <v>5130000</v>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 5 ảnh, 1 link nofollow (thêm link 500k)</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr"/>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 5,400,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
@@ -1154,14 +1174,18 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>6600000</v>
+        <v>6270000</v>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 5 ảnh</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n">
@@ -1173,14 +1197,18 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>4500000</v>
+        <v>4275000</v>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, 1 link nofollow (thêm link 500k)</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr"/>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 4,500,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
@@ -1192,14 +1220,18 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>7000000</v>
+        <v>6650000</v>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 5 ảnh</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -1211,14 +1243,18 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>7500000</v>
+        <v>7125000</v>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, không chèn link</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr"/>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -1230,14 +1266,18 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>9200000</v>
+        <v>8740000</v>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, mua 500k/link (3 link 1tr)</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr"/>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -1249,14 +1289,18 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>10500000</v>
+        <v>9975000</v>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, mua 500k/link (3 link 1tr)</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr"/>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 10,500,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -1268,14 +1312,18 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>7800000</v>
+        <v>7410000</v>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, 2 link nofollow</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
@@ -1287,16 +1335,16 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>2700000</v>
+        <v>2565000</v>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>700 từ, 3 ảnh, 2 link DOFOLLOW</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>DR 74 - dofollow, tốt cho SEO thương hiệu</t>
+          <t>700 từ, 3 ảnh, 2 link DOFOLLOW - DR 74</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 2,700,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -1310,16 +1358,16 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>3150000</v>
+        <v>2992000</v>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>1 link dofollow (thêm link 300k)</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>DR 69 - dofollow</t>
+          <t>1 link dofollow (thêm link 300k) - DR 69</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 3,150,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
         </is>
       </c>
     </row>
@@ -1333,14 +1381,18 @@
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>5000000</v>
+        <v>4750000</v>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, mua link riêng 5tr/link/3 tháng</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr"/>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 5,000,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -1352,14 +1404,18 @@
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>6000000</v>
+        <v>5700000</v>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, không chèn link</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr"/>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Trùng lần 1 (giá cũ 6,000,000đ) - đã trừ 5% DanaSEO. DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -1371,14 +1427,18 @@
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>9000000</v>
+        <v>8550000</v>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Dưới 1000 từ, dưới 3 ảnh, 1 link nofollow</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr"/>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>DanaSEO - đã trừ 5%</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -1399,7 +1459,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Nguồn: Rise Media</t>
+          <t>Nguồn: Rise Media (không phải DanaSEO - giữ nguyên giá vốn, KHÔNG áp công thức -5%)</t>
         </is>
       </c>
     </row>
@@ -1424,8 +1484,8 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1435,10 +1495,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Giá niêm yết trực tiếp từ nhà cung cấp báo (đã là giá tốt nhất Digicom đàm phán được, chưa gồm VAT 8% trừ khi ghi chú khác). Giá có thể thay đổi vào phút chót theo chính sách toà soạn - Digicom sẽ báo lại nếu có biến động trước khi khách chốt đăng.</t>
+          <t>Giá = giá vốn DanaSEO hiện hành TRỪ THÊM 5% (đúng công thức Hiếu chốt cho khách này). Với báo lấy nguồn từ NCC khác DanaSEO (không có mức giá DanaSEO để đối chiếu) - giữ nguyên giá vốn gốc, có ghi rõ nguồn. Dòng có ⚠ = TRÙNG outlet/vị trí đã gửi trong báo giá lần 1 nhưng giá SAU khi trừ 5% THẤP HƠN giá đã gửi lần 1 - cần Hiếu xác nhận có báo lại giá mới cho khách hay giữ nguyên giá cũ đã gửi.</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1548,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Nguồn: Xuyên Việt Media (đã là mức thấp nhất, dải giá NCC 35-50tr)</t>
+          <t>Nguồn: Xuyên Việt Media (không phải DanaSEO - giữ nguyên giá vốn, KHÔNG áp công thức -5%)</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1571,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Nguồn: Admicro (VCCorp) - đã gồm VAT 8%</t>
+          <t>Nguồn: Admicro/VCCorp (không phải DanaSEO - giữ nguyên giá vốn, đã gồm VAT 8%)</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1594,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Nguồn: Admicro (VCCorp) - chưa gồm 10% VAT + phí viết bài</t>
+          <t>Nguồn: Admicro/VCCorp (không phải DanaSEO - giữ nguyên giá vốn, chưa gồm 10% VAT + phí viết bài)</t>
         </is>
       </c>
     </row>

</xml_diff>